<commit_message>
Add more city monster
</commit_message>
<xml_diff>
--- a/doc/monster.xlsx
+++ b/doc/monster.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chaofan\AppData\Roaming\com.nesbox.tic\TIC-80\myproj\sts\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B28776EF-8CE1-440A-9AEC-AB92E9957D97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBDA663-525D-4CAD-9248-E465205205ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F23AF6A6-15E5-4CBC-A854-47F77E3852F2}"/>
   </bookViews>
@@ -926,10 +926,10 @@
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+      <c r="A27" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="1" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete act 3 events
</commit_message>
<xml_diff>
--- a/doc/monster.xlsx
+++ b/doc/monster.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chaofan\AppData\Roaming\com.nesbox.tic\TIC-80\myproj\sts\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0CF208C-3982-4156-B5A1-78BA61703674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D977408-D265-42FA-ACFF-B066CFEF3E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5010" yWindow="2100" windowWidth="18375" windowHeight="12690" xr2:uid="{F23AF6A6-15E5-4CBC-A854-47F77E3852F2}"/>
   </bookViews>
@@ -936,44 +936,44 @@
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
-        <v>0</v>
+      <c r="A20" s="6" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B22" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B23" s="4" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
         <v>30</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>